<commit_message>
Book directly on each place's official website instead of TheFork / GetYourGuide
- Official websites for ~75 places known with certainty (src/data/websites.ts);
  editors can add or fix a site in the admin screen (website field).
- Without a known site: the website relays through /api/reserve, which finds the
  official site via Google Places (with a key) and redirects; the preview opens the
  first search result for the place's official site.
- Excel export gains an "Site officiel" column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UXR8FGm153Rc6V8eWTCu3t
</commit_message>
<xml_diff>
--- a/exports/marco-base-de-donnees.xlsx
+++ b/exports/marco-base-de-donnees.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Annuaire des voies" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lieux'!$A$1:$P$197</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lieux'!$A$1:$Q$197</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rues racontées'!$A$1:$H$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Soirées'!$A$1:$F$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Casher-Halal'!$A$1:$E$8</definedName>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -665,43 +665,54 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>Sites officiels renseignés</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>COUNTIF(Lieux!P2:P1000,"https*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>Rues racontées</t>
         </is>
       </c>
-      <c r="B17" s="5">
+      <c r="B18" s="5">
         <f>COUNTA('Rues racontées'!A2:A1000)</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Lieux de soirée</t>
         </is>
       </c>
-      <c r="B18" s="5">
+      <c r="B19" s="5">
         <f>COUNTA(Soirées!C2:C1000)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Quartiers casher / halal</t>
         </is>
       </c>
-      <c r="B19" s="5">
+      <c r="B20" s="5">
         <f>COUNTA('Casher-Halal'!B2:B8)</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Voies dans l'annuaire</t>
         </is>
       </c>
-      <c r="B20" s="5">
+      <c r="B21" s="5">
         <f>COUNTA('Annuaire des voies'!A2:A10000)</f>
         <v/>
       </c>
@@ -720,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P197"/>
+  <dimension ref="A1:Q197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -738,7 +749,8 @@
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -819,6 +831,11 @@
       </c>
       <c r="P1" s="6" t="inlineStr">
         <is>
+          <t>Site officiel (réservation directe)</t>
+        </is>
+      </c>
+      <c r="Q1" s="6" t="inlineStr">
+        <is>
           <t>Identifiant</t>
         </is>
       </c>
@@ -885,6 +902,11 @@
       </c>
       <c r="P2" s="7" t="inlineStr">
         <is>
+          <t>https://www.angelina-paris.fr</t>
+        </is>
+      </c>
+      <c r="Q2" s="7" t="inlineStr">
+        <is>
           <t>angelina</t>
         </is>
       </c>
@@ -953,7 +975,8 @@
       <c r="O3" s="9" t="n">
         <v>2.3437</v>
       </c>
-      <c r="P3" s="9" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr"/>
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>pied-de-cochon</t>
         </is>
@@ -1021,6 +1044,11 @@
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
+          <t>https://www.ritzparis.com</t>
+        </is>
+      </c>
+      <c r="Q4" s="7" t="inlineStr">
+        <is>
           <t>bar-hemingway</t>
         </is>
       </c>
@@ -1089,7 +1117,8 @@
       <c r="O5" s="9" t="n">
         <v>2.3488</v>
       </c>
-      <c r="P5" s="9" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr"/>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>duc-lombards</t>
         </is>
@@ -1155,7 +1184,8 @@
       <c r="O6" s="7" t="n">
         <v>2.3375</v>
       </c>
-      <c r="P6" s="7" t="inlineStr">
+      <c r="P6" s="7" t="inlineStr"/>
+      <c r="Q6" s="7" t="inlineStr">
         <is>
           <t>palais-royal</t>
         </is>
@@ -1227,6 +1257,11 @@
       </c>
       <c r="P7" s="9" t="inlineStr">
         <is>
+          <t>https://www.kodawari-ramen.com</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
           <t>kodawari-tsukiji</t>
         </is>
       </c>
@@ -1295,7 +1330,8 @@
       <c r="O8" s="7" t="n">
         <v>2.3355</v>
       </c>
-      <c r="P8" s="7" t="inlineStr">
+      <c r="P8" s="7" t="inlineStr"/>
+      <c r="Q8" s="7" t="inlineStr">
         <is>
           <t>kunitoraya</t>
         </is>
@@ -1365,7 +1401,8 @@
       <c r="O9" s="9" t="n">
         <v>2.3478</v>
       </c>
-      <c r="P9" s="9" t="inlineStr">
+      <c r="P9" s="9" t="inlineStr"/>
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>dernier-bar</t>
         </is>
@@ -1437,6 +1474,11 @@
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
+          <t>https://www.grand-vefour.com</t>
+        </is>
+      </c>
+      <c r="Q10" s="7" t="inlineStr">
+        <is>
           <t>grand-vefour</t>
         </is>
       </c>
@@ -1506,6 +1548,11 @@
         <v>2.345</v>
       </c>
       <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>https://www.sainte-chapelle.fr</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>sainte-chapelle</t>
         </is>
@@ -1571,7 +1618,8 @@
       <c r="O12" s="7" t="n">
         <v>2.3405</v>
       </c>
-      <c r="P12" s="7" t="inlineStr">
+      <c r="P12" s="7" t="inlineStr"/>
+      <c r="Q12" s="7" t="inlineStr">
         <is>
           <t>vert-galant</t>
         </is>
@@ -1643,6 +1691,11 @@
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
+          <t>https://www.vedettesdupontneuf.com</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
           <t>vedettes-pont-neuf</t>
         </is>
       </c>
@@ -1713,6 +1766,11 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
+          <t>https://www.o-chateau.com</t>
+        </is>
+      </c>
+      <c r="Q14" s="7" t="inlineStr">
+        <is>
           <t>o-chateau</t>
         </is>
       </c>
@@ -1781,7 +1839,8 @@
       <c r="O15" s="9" t="n">
         <v>2.3391</v>
       </c>
-      <c r="P15" s="9" t="inlineStr">
+      <c r="P15" s="9" t="inlineStr"/>
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>daroco</t>
         </is>
@@ -1851,7 +1910,8 @@
       <c r="O16" s="7" t="n">
         <v>2.348</v>
       </c>
-      <c r="P16" s="7" t="inlineStr">
+      <c r="P16" s="7" t="inlineStr"/>
+      <c r="Q16" s="7" t="inlineStr">
         <is>
           <t>frenchie</t>
         </is>
@@ -1917,7 +1977,8 @@
       <c r="O17" s="9" t="n">
         <v>2.3398</v>
       </c>
-      <c r="P17" s="9" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr"/>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>galerie-vivienne</t>
         </is>
@@ -1989,6 +2050,11 @@
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
+          <t>https://www.legrandrex.com</t>
+        </is>
+      </c>
+      <c r="Q18" s="7" t="inlineStr">
+        <is>
           <t>grand-rex</t>
         </is>
       </c>
@@ -2057,7 +2123,8 @@
       <c r="O19" s="9" t="n">
         <v>2.3405</v>
       </c>
-      <c r="P19" s="9" t="inlineStr">
+      <c r="P19" s="9" t="inlineStr"/>
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>liza</t>
         </is>
@@ -2127,7 +2194,8 @@
       <c r="O20" s="7" t="n">
         <v>2.3396</v>
       </c>
-      <c r="P20" s="7" t="inlineStr">
+      <c r="P20" s="7" t="inlineStr"/>
+      <c r="Q20" s="7" t="inlineStr">
         <is>
           <t>mori-venice</t>
         </is>
@@ -2193,7 +2261,8 @@
       <c r="O21" s="9" t="n">
         <v>2.3417</v>
       </c>
-      <c r="P21" s="9" t="inlineStr">
+      <c r="P21" s="9" t="inlineStr"/>
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>passage-panoramas</t>
         </is>
@@ -2265,6 +2334,11 @@
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
+          <t>https://www.bigmammagroup.com</t>
+        </is>
+      </c>
+      <c r="Q22" s="7" t="inlineStr">
+        <is>
           <t>pizzeria-popolare</t>
         </is>
       </c>
@@ -2333,7 +2407,8 @@
       <c r="O23" s="9" t="n">
         <v>2.3419</v>
       </c>
-      <c r="P23" s="9" t="inlineStr">
+      <c r="P23" s="9" t="inlineStr"/>
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>racines</t>
         </is>
@@ -2403,7 +2478,8 @@
       <c r="O24" s="7" t="n">
         <v>2.3391</v>
       </c>
-      <c r="P24" s="7" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr"/>
+      <c r="Q24" s="7" t="inlineStr">
         <is>
           <t>bnf-richelieu</t>
         </is>
@@ -2469,7 +2545,8 @@
       <c r="O25" s="9" t="n">
         <v>2.3657</v>
       </c>
-      <c r="P25" s="9" t="inlineStr">
+      <c r="P25" s="9" t="inlineStr"/>
+      <c r="Q25" s="9" t="inlineStr">
         <is>
           <t>boot-cafe</t>
         </is>
@@ -2540,6 +2617,11 @@
         <v>2.3625</v>
       </c>
       <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t>https://breizhcafe.com</t>
+        </is>
+      </c>
+      <c r="Q26" s="7" t="inlineStr">
         <is>
           <t>breizh-cafe</t>
         </is>
@@ -2605,7 +2687,8 @@
       <c r="O27" s="9" t="n">
         <v>2.3637</v>
       </c>
-      <c r="P27" s="9" t="inlineStr">
+      <c r="P27" s="9" t="inlineStr"/>
+      <c r="Q27" s="9" t="inlineStr">
         <is>
           <t>candelaria</t>
         </is>
@@ -2675,7 +2758,8 @@
       <c r="O28" s="7" t="n">
         <v>2.362</v>
       </c>
-      <c r="P28" s="7" t="inlineStr">
+      <c r="P28" s="7" t="inlineStr"/>
+      <c r="Q28" s="7" t="inlineStr">
         <is>
           <t>alain-miam-miam</t>
         </is>
@@ -2747,6 +2831,11 @@
       </c>
       <c r="P29" s="9" t="inlineStr">
         <is>
+          <t>https://www.chezjanou.com</t>
+        </is>
+      </c>
+      <c r="Q29" s="9" t="inlineStr">
+        <is>
           <t>chez-janou</t>
         </is>
       </c>
@@ -2815,7 +2904,8 @@
       <c r="O30" s="7" t="n">
         <v>2.3616</v>
       </c>
-      <c r="P30" s="7" t="inlineStr">
+      <c r="P30" s="7" t="inlineStr"/>
+      <c r="Q30" s="7" t="inlineStr">
         <is>
           <t>chez-omar</t>
         </is>
@@ -2881,7 +2971,8 @@
       <c r="O31" s="9" t="n">
         <v>2.3534</v>
       </c>
-      <c r="P31" s="9" t="inlineStr">
+      <c r="P31" s="9" t="inlineStr"/>
+      <c r="Q31" s="9" t="inlineStr">
         <is>
           <t>jardin-anne-frank</t>
         </is>
@@ -2951,7 +3042,8 @@
       <c r="O32" s="7" t="n">
         <v>2.3547</v>
       </c>
-      <c r="P32" s="7" t="inlineStr">
+      <c r="P32" s="7" t="inlineStr"/>
+      <c r="Q32" s="7" t="inlineStr">
         <is>
           <t>cafe-des-chats</t>
         </is>
@@ -3017,7 +3109,8 @@
       <c r="O33" s="9" t="n">
         <v>2.3662</v>
       </c>
-      <c r="P33" s="9" t="inlineStr">
+      <c r="P33" s="9" t="inlineStr"/>
+      <c r="Q33" s="9" t="inlineStr">
         <is>
           <t>mary-celeste</t>
         </is>
@@ -3087,7 +3180,8 @@
       <c r="O34" s="7" t="n">
         <v>2.3622</v>
       </c>
-      <c r="P34" s="7" t="inlineStr">
+      <c r="P34" s="7" t="inlineStr"/>
+      <c r="Q34" s="7" t="inlineStr">
         <is>
           <t>enfants-du-marche</t>
         </is>
@@ -3157,7 +3251,8 @@
       <c r="O35" s="9" t="n">
         <v>2.362</v>
       </c>
-      <c r="P35" s="9" t="inlineStr">
+      <c r="P35" s="9" t="inlineStr"/>
+      <c r="Q35" s="9" t="inlineStr">
         <is>
           <t>enfants-rouges</t>
         </is>
@@ -3225,6 +3320,11 @@
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
+          <t>https://www.carnavalet.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q36" s="7" t="inlineStr">
+        <is>
           <t>carnavalet</t>
         </is>
       </c>
@@ -3295,6 +3395,11 @@
       </c>
       <c r="P37" s="9" t="inlineStr">
         <is>
+          <t>https://www.chassenature.org</t>
+        </is>
+      </c>
+      <c r="Q37" s="9" t="inlineStr">
+        <is>
           <t>musee-chasse</t>
         </is>
       </c>
@@ -3365,6 +3470,11 @@
       </c>
       <c r="P38" s="7" t="inlineStr">
         <is>
+          <t>https://www.arts-et-metiers.net</t>
+        </is>
+      </c>
+      <c r="Q38" s="7" t="inlineStr">
+        <is>
           <t>arts-et-metiers</t>
         </is>
       </c>
@@ -3435,6 +3545,11 @@
       </c>
       <c r="P39" s="9" t="inlineStr">
         <is>
+          <t>https://www.benoit-paris.com</t>
+        </is>
+      </c>
+      <c r="Q39" s="9" t="inlineStr">
+        <is>
           <t>benoit</t>
         </is>
       </c>
@@ -3503,7 +3618,8 @@
       <c r="O40" s="7" t="n">
         <v>2.3553</v>
       </c>
-      <c r="P40" s="7" t="inlineStr">
+      <c r="P40" s="7" t="inlineStr"/>
+      <c r="Q40" s="7" t="inlineStr">
         <is>
           <t>chez-julien</t>
         </is>
@@ -3573,7 +3689,8 @@
       <c r="O41" s="9" t="n">
         <v>2.3538</v>
       </c>
-      <c r="P41" s="9" t="inlineStr">
+      <c r="P41" s="9" t="inlineStr"/>
+      <c r="Q41" s="9" t="inlineStr">
         <is>
           <t>grand-coeur</t>
         </is>
@@ -3647,7 +3764,8 @@
       <c r="O42" s="7" t="n">
         <v>2.3591</v>
       </c>
-      <c r="P42" s="7" t="inlineStr">
+      <c r="P42" s="7" t="inlineStr"/>
+      <c r="Q42" s="7" t="inlineStr">
         <is>
           <t>as-du-fallafel</t>
         </is>
@@ -3718,6 +3836,11 @@
         <v>2.3547</v>
       </c>
       <c r="P43" s="9" t="inlineStr">
+        <is>
+          <t>https://www.lacuisineparis.com</t>
+        </is>
+      </c>
+      <c r="Q43" s="9" t="inlineStr">
         <is>
           <t>la-cuisine-paris</t>
         </is>
@@ -3785,6 +3908,11 @@
       </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
+          <t>https://www.maisonsvictorhugo.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q44" s="7" t="inlineStr">
+        <is>
           <t>maison-victor-hugo</t>
         </is>
       </c>
@@ -3853,7 +3981,8 @@
       <c r="O45" s="9" t="n">
         <v>2.3471</v>
       </c>
-      <c r="P45" s="9" t="inlineStr">
+      <c r="P45" s="9" t="inlineStr"/>
+      <c r="Q45" s="9" t="inlineStr">
         <is>
           <t>marche-aux-fleurs</t>
         </is>
@@ -3923,7 +4052,8 @@
       <c r="O46" s="7" t="n">
         <v>2.3587</v>
       </c>
-      <c r="P46" s="7" t="inlineStr">
+      <c r="P46" s="7" t="inlineStr"/>
+      <c r="Q46" s="7" t="inlineStr">
         <is>
           <t>miznon</t>
         </is>
@@ -3994,6 +4124,11 @@
         <v>2.3622</v>
       </c>
       <c r="P47" s="9" t="inlineStr">
+        <is>
+          <t>https://www.museedelamagie.com</t>
+        </is>
+      </c>
+      <c r="Q47" s="9" t="inlineStr">
         <is>
           <t>musee-magie</t>
         </is>
@@ -4059,7 +4194,8 @@
       <c r="O48" s="7" t="n">
         <v>2.3642</v>
       </c>
-      <c r="P48" s="7" t="inlineStr">
+      <c r="P48" s="7" t="inlineStr"/>
+      <c r="Q48" s="7" t="inlineStr">
         <is>
           <t>hotel-sully</t>
         </is>
@@ -4125,7 +4261,8 @@
       <c r="O49" s="9" t="n">
         <v>2.3614</v>
       </c>
-      <c r="P49" s="9" t="inlineStr">
+      <c r="P49" s="9" t="inlineStr"/>
+      <c r="Q49" s="9" t="inlineStr">
         <is>
           <t>village-saint-paul</t>
         </is>
@@ -4191,7 +4328,8 @@
       <c r="O50" s="7" t="n">
         <v>2.3527</v>
       </c>
-      <c r="P50" s="7" t="inlineStr">
+      <c r="P50" s="7" t="inlineStr"/>
+      <c r="Q50" s="7" t="inlineStr">
         <is>
           <t>arenes-lutece</t>
         </is>
@@ -4261,7 +4399,8 @@
       <c r="O51" s="9" t="n">
         <v>2.3497</v>
       </c>
-      <c r="P51" s="9" t="inlineStr">
+      <c r="P51" s="9" t="inlineStr"/>
+      <c r="Q51" s="9" t="inlineStr">
         <is>
           <t>bowling-mouffetard</t>
         </is>
@@ -4331,7 +4470,8 @@
       <c r="O52" s="7" t="n">
         <v>2.3432</v>
       </c>
-      <c r="P52" s="7" t="inlineStr">
+      <c r="P52" s="7" t="inlineStr"/>
+      <c r="Q52" s="7" t="inlineStr">
         <is>
           <t>nouvelle-mairie</t>
         </is>
@@ -4397,7 +4537,8 @@
       <c r="O53" s="9" t="n">
         <v>2.3464</v>
       </c>
-      <c r="P53" s="9" t="inlineStr">
+      <c r="P53" s="9" t="inlineStr"/>
+      <c r="Q53" s="9" t="inlineStr">
         <is>
           <t>caveau-huchette</t>
         </is>
@@ -4469,6 +4610,11 @@
       </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
+          <t>https://www.paris-pantheon.fr</t>
+        </is>
+      </c>
+      <c r="Q54" s="7" t="inlineStr">
+        <is>
           <t>pantheon-coupole</t>
         </is>
       </c>
@@ -4537,7 +4683,8 @@
       <c r="O55" s="9" t="n">
         <v>2.3602</v>
       </c>
-      <c r="P55" s="9" t="inlineStr">
+      <c r="P55" s="9" t="inlineStr"/>
+      <c r="Q55" s="9" t="inlineStr">
         <is>
           <t>tango-quai</t>
         </is>
@@ -4609,6 +4756,11 @@
       </c>
       <c r="P56" s="7" t="inlineStr">
         <is>
+          <t>https://tourdargent.com</t>
+        </is>
+      </c>
+      <c r="Q56" s="7" t="inlineStr">
+        <is>
           <t>tour-argent</t>
         </is>
       </c>
@@ -4677,7 +4829,8 @@
       <c r="O57" s="9" t="n">
         <v>2.3464</v>
       </c>
-      <c r="P57" s="9" t="inlineStr">
+      <c r="P57" s="9" t="inlineStr"/>
+      <c r="Q57" s="9" t="inlineStr">
         <is>
           <t>petit-prince</t>
         </is>
@@ -4747,7 +4900,8 @@
       <c r="O58" s="7" t="n">
         <v>2.3408</v>
       </c>
-      <c r="P58" s="7" t="inlineStr">
+      <c r="P58" s="7" t="inlineStr"/>
+      <c r="Q58" s="7" t="inlineStr">
         <is>
           <t>les-papilles</t>
         </is>
@@ -4819,6 +4973,11 @@
       </c>
       <c r="P59" s="9" t="inlineStr">
         <is>
+          <t>https://www.musee-moyenage.fr</t>
+        </is>
+      </c>
+      <c r="Q59" s="9" t="inlineStr">
+        <is>
           <t>cluny</t>
         </is>
       </c>
@@ -4887,7 +5046,8 @@
       <c r="O60" s="7" t="n">
         <v>2.3601</v>
       </c>
-      <c r="P60" s="7" t="inlineStr">
+      <c r="P60" s="7" t="inlineStr"/>
+      <c r="Q60" s="7" t="inlineStr">
         <is>
           <t>menagerie</t>
         </is>
@@ -4957,7 +5117,8 @@
       <c r="O61" s="9" t="n">
         <v>2.3531</v>
       </c>
-      <c r="P61" s="9" t="inlineStr">
+      <c r="P61" s="9" t="inlineStr"/>
+      <c r="Q61" s="9" t="inlineStr">
         <is>
           <t>piscine-pontoise</t>
         </is>
@@ -5031,7 +5192,8 @@
       <c r="O62" s="7" t="n">
         <v>2.3551</v>
       </c>
-      <c r="P62" s="7" t="inlineStr">
+      <c r="P62" s="7" t="inlineStr"/>
+      <c r="Q62" s="7" t="inlineStr">
         <is>
           <t>grande-mosquee-resto</t>
         </is>
@@ -5097,7 +5259,8 @@
       <c r="O63" s="9" t="n">
         <v>2.3553</v>
       </c>
-      <c r="P63" s="9" t="inlineStr">
+      <c r="P63" s="9" t="inlineStr"/>
+      <c r="Q63" s="9" t="inlineStr">
         <is>
           <t>mosquee-the</t>
         </is>
@@ -5165,6 +5328,11 @@
       </c>
       <c r="P64" s="7" t="inlineStr">
         <is>
+          <t>https://shakespeareandcompany.com</t>
+        </is>
+      </c>
+      <c r="Q64" s="7" t="inlineStr">
+        <is>
           <t>shakespeare</t>
         </is>
       </c>
@@ -5234,6 +5402,11 @@
         <v>2.3413</v>
       </c>
       <c r="P65" s="9" t="inlineStr">
+        <is>
+          <t>https://www.bouillonracine.com</t>
+        </is>
+      </c>
+      <c r="Q65" s="9" t="inlineStr">
         <is>
           <t>bouillon-racine</t>
         </is>
@@ -5301,6 +5474,11 @@
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
+          <t>https://cafedeflore.fr</t>
+        </is>
+      </c>
+      <c r="Q66" s="7" t="inlineStr">
+        <is>
           <t>flore</t>
         </is>
       </c>
@@ -5365,7 +5543,8 @@
       <c r="O67" s="9" t="n">
         <v>2.3387</v>
       </c>
-      <c r="P67" s="9" t="inlineStr">
+      <c r="P67" s="9" t="inlineStr"/>
+      <c r="Q67" s="9" t="inlineStr">
         <is>
           <t>cour-commerce</t>
         </is>
@@ -5435,7 +5614,8 @@
       <c r="O68" s="7" t="n">
         <v>2.3354</v>
       </c>
-      <c r="P68" s="7" t="inlineStr">
+      <c r="P68" s="7" t="inlineStr"/>
+      <c r="Q68" s="7" t="inlineStr">
         <is>
           <t>bon-saint-pourcain</t>
         </is>
@@ -5505,7 +5685,8 @@
       <c r="O69" s="9" t="n">
         <v>2.3389</v>
       </c>
-      <c r="P69" s="9" t="inlineStr">
+      <c r="P69" s="9" t="inlineStr"/>
+      <c r="Q69" s="9" t="inlineStr">
         <is>
           <t>comptoir-relais</t>
         </is>
@@ -5577,6 +5758,11 @@
       </c>
       <c r="P70" s="7" t="inlineStr">
         <is>
+          <t>https://www.procope.com</t>
+        </is>
+      </c>
+      <c r="Q70" s="7" t="inlineStr">
+        <is>
           <t>procope</t>
         </is>
       </c>
@@ -5646,6 +5832,11 @@
         <v>2.3329</v>
       </c>
       <c r="P71" s="9" t="inlineStr">
+        <is>
+          <t>https://www.relaisentrecote.fr</t>
+        </is>
+      </c>
+      <c r="Q71" s="9" t="inlineStr">
         <is>
           <t>relais-entrecote</t>
         </is>
@@ -5713,6 +5904,11 @@
       </c>
       <c r="P72" s="7" t="inlineStr">
         <is>
+          <t>https://www.lesdeuxmagots.fr</t>
+        </is>
+      </c>
+      <c r="Q72" s="7" t="inlineStr">
+        <is>
           <t>deux-magots</t>
         </is>
       </c>
@@ -5779,6 +5975,11 @@
       </c>
       <c r="P73" s="9" t="inlineStr">
         <is>
+          <t>https://www.zadkine.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q73" s="9" t="inlineStr">
+        <is>
           <t>zadkine</t>
         </is>
       </c>
@@ -5847,7 +6048,8 @@
       <c r="O74" s="7" t="n">
         <v>2.3401</v>
       </c>
-      <c r="P74" s="7" t="inlineStr">
+      <c r="P74" s="7" t="inlineStr"/>
+      <c r="Q74" s="7" t="inlineStr">
         <is>
           <t>polidor</t>
         </is>
@@ -5917,7 +6119,8 @@
       <c r="O75" s="9" t="n">
         <v>2.3371</v>
       </c>
-      <c r="P75" s="9" t="inlineStr">
+      <c r="P75" s="9" t="inlineStr"/>
+      <c r="Q75" s="9" t="inlineStr">
         <is>
           <t>semilla</t>
         </is>
@@ -5989,6 +6192,11 @@
       </c>
       <c r="P76" s="7" t="inlineStr">
         <is>
+          <t>https://www.alain-passard.com</t>
+        </is>
+      </c>
+      <c r="Q76" s="7" t="inlineStr">
+        <is>
           <t>arpege</t>
         </is>
       </c>
@@ -6057,7 +6265,8 @@
       <c r="O77" s="9" t="n">
         <v>2.3014</v>
       </c>
-      <c r="P77" s="9" t="inlineStr">
+      <c r="P77" s="9" t="inlineStr"/>
+      <c r="Q77" s="9" t="inlineStr">
         <is>
           <t>cafe-constant</t>
         </is>
@@ -6123,7 +6332,8 @@
       <c r="O78" s="7" t="n">
         <v>2.3252</v>
       </c>
-      <c r="P78" s="7" t="inlineStr">
+      <c r="P78" s="7" t="inlineStr"/>
+      <c r="Q78" s="7" t="inlineStr">
         <is>
           <t>deyrolle</t>
         </is>
@@ -6193,7 +6403,8 @@
       <c r="O79" s="9" t="n">
         <v>2.3037</v>
       </c>
-      <c r="P79" s="9" t="inlineStr">
+      <c r="P79" s="9" t="inlineStr"/>
+      <c r="Q79" s="9" t="inlineStr">
         <is>
           <t>ami-jean</t>
         </is>
@@ -6263,7 +6474,8 @@
       <c r="O80" s="7" t="n">
         <v>2.302</v>
       </c>
-      <c r="P80" s="7" t="inlineStr">
+      <c r="P80" s="7" t="inlineStr"/>
+      <c r="Q80" s="7" t="inlineStr">
         <is>
           <t>les-cocottes</t>
         </is>
@@ -6335,6 +6547,11 @@
       </c>
       <c r="P81" s="9" t="inlineStr">
         <is>
+          <t>https://www.musee-rodin.fr</t>
+        </is>
+      </c>
+      <c r="Q81" s="9" t="inlineStr">
+        <is>
           <t>musee-rodin</t>
         </is>
       </c>
@@ -6405,6 +6622,11 @@
       </c>
       <c r="P82" s="7" t="inlineStr">
         <is>
+          <t>https://www.musee-egouts.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q82" s="7" t="inlineStr">
+        <is>
           <t>egouts</t>
         </is>
       </c>
@@ -6475,6 +6697,11 @@
       </c>
       <c r="P83" s="9" t="inlineStr">
         <is>
+          <t>https://www.toureiffel.paris</t>
+        </is>
+      </c>
+      <c r="Q83" s="9" t="inlineStr">
+        <is>
           <t>tour-eiffel-escaliers</t>
         </is>
       </c>
@@ -6543,7 +6770,8 @@
       <c r="O84" s="7" t="n">
         <v>2.3044</v>
       </c>
-      <c r="P84" s="7" t="inlineStr">
+      <c r="P84" s="7" t="inlineStr"/>
+      <c r="Q84" s="7" t="inlineStr">
         <is>
           <t>chez-savy</t>
         </is>
@@ -6615,6 +6843,11 @@
       </c>
       <c r="P85" s="9" t="inlineStr">
         <is>
+          <t>https://www.le-laurent.com</t>
+        </is>
+      </c>
+      <c r="Q85" s="9" t="inlineStr">
+        <is>
           <t>laurent</t>
         </is>
       </c>
@@ -6683,7 +6916,8 @@
       <c r="O86" s="7" t="n">
         <v>2.3099</v>
       </c>
-      <c r="P86" s="7" t="inlineStr">
+      <c r="P86" s="7" t="inlineStr"/>
+      <c r="Q86" s="7" t="inlineStr">
         <is>
           <t>boeuf-sur-le-toit</t>
         </is>
@@ -6755,6 +6989,11 @@
       </c>
       <c r="P87" s="9" t="inlineStr">
         <is>
+          <t>https://www.musee-jacquemart-andre.com</t>
+        </is>
+      </c>
+      <c r="Q87" s="9" t="inlineStr">
+        <is>
           <t>jacquemart-andre</t>
         </is>
       </c>
@@ -6825,6 +7064,11 @@
       </c>
       <c r="P88" s="7" t="inlineStr">
         <is>
+          <t>https://madparis.fr</t>
+        </is>
+      </c>
+      <c r="Q88" s="7" t="inlineStr">
+        <is>
           <t>nissim-camondo</t>
         </is>
       </c>
@@ -6893,7 +7137,8 @@
       <c r="O89" s="9" t="n">
         <v>2.3163</v>
       </c>
-      <c r="P89" s="9" t="inlineStr">
+      <c r="P89" s="9" t="inlineStr"/>
+      <c r="Q89" s="9" t="inlineStr">
         <is>
           <t>pavillon-ledoyen</t>
         </is>
@@ -6959,7 +7204,8 @@
       <c r="O90" s="7" t="n">
         <v>2.3148</v>
       </c>
-      <c r="P90" s="7" t="inlineStr">
+      <c r="P90" s="7" t="inlineStr"/>
+      <c r="Q90" s="7" t="inlineStr">
         <is>
           <t>petit-palais</t>
         </is>
@@ -7031,6 +7277,11 @@
       </c>
       <c r="P91" s="9" t="inlineStr">
         <is>
+          <t>https://www.paris-arc-de-triomphe.fr</t>
+        </is>
+      </c>
+      <c r="Q91" s="9" t="inlineStr">
+        <is>
           <t>arc-triomphe-toit</t>
         </is>
       </c>
@@ -7101,6 +7352,11 @@
       </c>
       <c r="P92" s="7" t="inlineStr">
         <is>
+          <t>https://www.bouillon-chartier.com</t>
+        </is>
+      </c>
+      <c r="Q92" s="7" t="inlineStr">
+        <is>
           <t>bouillon-chartier</t>
         </is>
       </c>
@@ -7169,7 +7425,8 @@
       <c r="O93" s="9" t="n">
         <v>2.3392</v>
       </c>
-      <c r="P93" s="9" t="inlineStr">
+      <c r="P93" s="9" t="inlineStr"/>
+      <c r="Q93" s="9" t="inlineStr">
         <is>
           <t>hotel-amour</t>
         </is>
@@ -7239,7 +7496,8 @@
       <c r="O94" s="7" t="n">
         <v>2.3375</v>
       </c>
-      <c r="P94" s="7" t="inlineStr">
+      <c r="P94" s="7" t="inlineStr"/>
+      <c r="Q94" s="7" t="inlineStr">
         <is>
           <t>bon-georges</t>
         </is>
@@ -7309,7 +7567,8 @@
       <c r="O95" s="9" t="n">
         <v>2.3431</v>
       </c>
-      <c r="P95" s="9" t="inlineStr">
+      <c r="P95" s="9" t="inlineStr"/>
+      <c r="Q95" s="9" t="inlineStr">
         <is>
           <t>pates-vivantes</t>
         </is>
@@ -7380,6 +7639,11 @@
         <v>2.3421</v>
       </c>
       <c r="P96" s="7" t="inlineStr">
+        <is>
+          <t>https://www.grevin-paris.com</t>
+        </is>
+      </c>
+      <c r="Q96" s="7" t="inlineStr">
         <is>
           <t>musee-grevin</t>
         </is>
@@ -7447,6 +7711,11 @@
       </c>
       <c r="P97" s="9" t="inlineStr">
         <is>
+          <t>https://museevieromantique.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q97" s="9" t="inlineStr">
+        <is>
           <t>vie-romantique</t>
         </is>
       </c>
@@ -7517,6 +7786,11 @@
       </c>
       <c r="P98" s="7" t="inlineStr">
         <is>
+          <t>https://www.fragonard.com</t>
+        </is>
+      </c>
+      <c r="Q98" s="7" t="inlineStr">
+        <is>
           <t>fragonard</t>
         </is>
       </c>
@@ -7587,6 +7861,11 @@
       </c>
       <c r="P99" s="9" t="inlineStr">
         <is>
+          <t>https://www.bigmammagroup.com</t>
+        </is>
+      </c>
+      <c r="Q99" s="9" t="inlineStr">
+        <is>
           <t>pink-mamma</t>
         </is>
       </c>
@@ -7657,6 +7936,11 @@
       </c>
       <c r="P100" s="7" t="inlineStr">
         <is>
+          <t>https://www.operadeparis.fr</t>
+        </is>
+      </c>
+      <c r="Q100" s="7" t="inlineStr">
+        <is>
           <t>opera-garnier</t>
         </is>
       </c>
@@ -7727,6 +8011,11 @@
       </c>
       <c r="P101" s="9" t="inlineStr">
         <is>
+          <t>https://www.bouillon-julien.com</t>
+        </is>
+      </c>
+      <c r="Q101" s="9" t="inlineStr">
+        <is>
           <t>bouillon-julien</t>
         </is>
       </c>
@@ -7795,7 +8084,8 @@
       <c r="O102" s="7" t="n">
         <v>2.3521</v>
       </c>
-      <c r="P102" s="7" t="inlineStr">
+      <c r="P102" s="7" t="inlineStr"/>
+      <c r="Q102" s="7" t="inlineStr">
         <is>
           <t>chez-michel</t>
         </is>
@@ -7863,6 +8153,11 @@
       </c>
       <c r="P103" s="9" t="inlineStr">
         <is>
+          <t>https://dupainetdesidees.com</t>
+        </is>
+      </c>
+      <c r="Q103" s="9" t="inlineStr">
+        <is>
           <t>pain-idees</t>
         </is>
       </c>
@@ -7929,6 +8224,11 @@
       </c>
       <c r="P104" s="7" t="inlineStr">
         <is>
+          <t>https://holybellycafe.com</t>
+        </is>
+      </c>
+      <c r="Q104" s="7" t="inlineStr">
+        <is>
           <t>holybelly</t>
         </is>
       </c>
@@ -7993,7 +8293,8 @@
       <c r="O105" s="9" t="n">
         <v>2.3649</v>
       </c>
-      <c r="P105" s="9" t="inlineStr">
+      <c r="P105" s="9" t="inlineStr"/>
+      <c r="Q105" s="9" t="inlineStr">
         <is>
           <t>hotel-du-nord</t>
         </is>
@@ -8059,7 +8360,8 @@
       <c r="O106" s="7" t="n">
         <v>2.3662</v>
       </c>
-      <c r="P106" s="7" t="inlineStr">
+      <c r="P106" s="7" t="inlineStr"/>
+      <c r="Q106" s="7" t="inlineStr">
         <is>
           <t>comptoir-general</t>
         </is>
@@ -8129,7 +8431,8 @@
       <c r="O107" s="9" t="n">
         <v>2.3706</v>
       </c>
-      <c r="P107" s="9" t="inlineStr">
+      <c r="P107" s="9" t="inlineStr"/>
+      <c r="Q107" s="9" t="inlineStr">
         <is>
           <t>le-galopin</t>
         </is>
@@ -8195,7 +8498,8 @@
       <c r="O108" s="7" t="n">
         <v>2.354</v>
       </c>
-      <c r="P108" s="7" t="inlineStr">
+      <c r="P108" s="7" t="inlineStr"/>
+      <c r="Q108" s="7" t="inlineStr">
         <is>
           <t>syndicat</t>
         </is>
@@ -8261,7 +8565,8 @@
       <c r="O109" s="9" t="n">
         <v>2.3653</v>
       </c>
-      <c r="P109" s="9" t="inlineStr">
+      <c r="P109" s="9" t="inlineStr"/>
+      <c r="Q109" s="9" t="inlineStr">
         <is>
           <t>ten-belles</t>
         </is>
@@ -8331,7 +8636,8 @@
       <c r="O110" s="7" t="n">
         <v>2.3541</v>
       </c>
-      <c r="P110" s="7" t="inlineStr">
+      <c r="P110" s="7" t="inlineStr"/>
+      <c r="Q110" s="7" t="inlineStr">
         <is>
           <t>urfa-durum</t>
         </is>
@@ -8403,6 +8709,11 @@
       </c>
       <c r="P111" s="9" t="inlineStr">
         <is>
+          <t>https://www.atelier-lumieres.com</t>
+        </is>
+      </c>
+      <c r="Q111" s="9" t="inlineStr">
+        <is>
           <t>atelier-lumieres</t>
         </is>
       </c>
@@ -8471,7 +8782,8 @@
       <c r="O112" s="7" t="n">
         <v>2.3702</v>
       </c>
-      <c r="P112" s="7" t="inlineStr">
+      <c r="P112" s="7" t="inlineStr"/>
+      <c r="Q112" s="7" t="inlineStr">
         <is>
           <t>deux-amis</t>
         </is>
@@ -8541,7 +8853,8 @@
       <c r="O113" s="9" t="n">
         <v>2.3845</v>
       </c>
-      <c r="P113" s="9" t="inlineStr">
+      <c r="P113" s="9" t="inlineStr"/>
+      <c r="Q113" s="9" t="inlineStr">
         <is>
           <t>bistrot-paul-bert</t>
         </is>
@@ -8613,6 +8926,11 @@
       </c>
       <c r="P114" s="7" t="inlineStr">
         <is>
+          <t>https://www.clamato-charonne.fr</t>
+        </is>
+      </c>
+      <c r="Q114" s="7" t="inlineStr">
+        <is>
           <t>clamato</t>
         </is>
       </c>
@@ -8681,7 +8999,8 @@
       <c r="O115" s="9" t="n">
         <v>2.3666</v>
       </c>
-      <c r="P115" s="9" t="inlineStr">
+      <c r="P115" s="9" t="inlineStr"/>
+      <c r="Q115" s="9" t="inlineStr">
         <is>
           <t>clown-bar</t>
         </is>
@@ -8752,6 +9071,11 @@
         <v>2.3712</v>
       </c>
       <c r="P116" s="7" t="inlineStr">
+        <is>
+          <t>https://www.lechateaubriand.net</t>
+        </is>
+      </c>
+      <c r="Q116" s="7" t="inlineStr">
         <is>
           <t>chateaubriand</t>
         </is>
@@ -8819,6 +9143,11 @@
       </c>
       <c r="P117" s="9" t="inlineStr">
         <is>
+          <t>https://leperchoir.fr</t>
+        </is>
+      </c>
+      <c r="Q117" s="9" t="inlineStr">
+        <is>
           <t>perchoir</t>
         </is>
       </c>
@@ -8887,7 +9216,8 @@
       <c r="O118" s="7" t="n">
         <v>2.3771</v>
       </c>
-      <c r="P118" s="7" t="inlineStr">
+      <c r="P118" s="7" t="inlineStr"/>
+      <c r="Q118" s="7" t="inlineStr">
         <is>
           <t>le-president</t>
         </is>
@@ -8957,7 +9287,8 @@
       <c r="O119" s="9" t="n">
         <v>2.3806</v>
       </c>
-      <c r="P119" s="9" t="inlineStr">
+      <c r="P119" s="9" t="inlineStr"/>
+      <c r="Q119" s="9" t="inlineStr">
         <is>
           <t>le-servan</t>
         </is>
@@ -9027,7 +9358,8 @@
       <c r="O120" s="7" t="n">
         <v>2.3805</v>
       </c>
-      <c r="P120" s="7" t="inlineStr">
+      <c r="P120" s="7" t="inlineStr"/>
+      <c r="Q120" s="7" t="inlineStr">
         <is>
           <t>musee-edith-piaf</t>
         </is>
@@ -9099,6 +9431,11 @@
       </c>
       <c r="P121" s="9" t="inlineStr">
         <is>
+          <t>https://www.parisvelosympa.com</t>
+        </is>
+      </c>
+      <c r="Q121" s="9" t="inlineStr">
+        <is>
           <t>velo-paris-sympa</t>
         </is>
       </c>
@@ -9168,6 +9505,11 @@
         <v>2.381</v>
       </c>
       <c r="P122" s="7" t="inlineStr">
+        <is>
+          <t>https://www.septime-charonne.fr</t>
+        </is>
+      </c>
+      <c r="Q122" s="7" t="inlineStr">
         <is>
           <t>septime</t>
         </is>
@@ -9233,7 +9575,8 @@
       <c r="O123" s="9" t="n">
         <v>2.376</v>
       </c>
-      <c r="P123" s="9" t="inlineStr">
+      <c r="P123" s="9" t="inlineStr"/>
+      <c r="Q123" s="9" t="inlineStr">
         <is>
           <t>coulee-verte</t>
         </is>
@@ -9299,7 +9642,8 @@
       <c r="O124" s="7" t="n">
         <v>2.378</v>
       </c>
-      <c r="P124" s="7" t="inlineStr">
+      <c r="P124" s="7" t="inlineStr"/>
+      <c r="Q124" s="7" t="inlineStr">
         <is>
           <t>baron-rouge</t>
         </is>
@@ -9369,7 +9713,8 @@
       <c r="O125" s="9" t="n">
         <v>2.3771</v>
       </c>
-      <c r="P125" s="9" t="inlineStr">
+      <c r="P125" s="9" t="inlineStr"/>
+      <c r="Q125" s="9" t="inlineStr">
         <is>
           <t>square-trousseau</t>
         </is>
@@ -9441,6 +9786,11 @@
       </c>
       <c r="P126" s="7" t="inlineStr">
         <is>
+          <t>https://www.le-train-bleu.com</t>
+        </is>
+      </c>
+      <c r="Q126" s="7" t="inlineStr">
+        <is>
           <t>train-bleu</t>
         </is>
       </c>
@@ -9511,6 +9861,11 @@
       </c>
       <c r="P127" s="9" t="inlineStr">
         <is>
+          <t>https://arts-forains.com</t>
+        </is>
+      </c>
+      <c r="Q127" s="9" t="inlineStr">
+        <is>
           <t>arts-forains</t>
         </is>
       </c>
@@ -9581,6 +9936,11 @@
       </c>
       <c r="P128" s="7" t="inlineStr">
         <is>
+          <t>https://www.parczoologiquedeparis.fr</t>
+        </is>
+      </c>
+      <c r="Q128" s="7" t="inlineStr">
+        <is>
           <t>zoo-vincennes</t>
         </is>
       </c>
@@ -9649,7 +10009,8 @@
       <c r="O129" s="9" t="n">
         <v>2.3774</v>
       </c>
-      <c r="P129" s="9" t="inlineStr">
+      <c r="P129" s="9" t="inlineStr"/>
+      <c r="Q129" s="9" t="inlineStr">
         <is>
           <t>table-verjus</t>
         </is>
@@ -9719,7 +10080,8 @@
       <c r="O130" s="7" t="n">
         <v>2.3505</v>
       </c>
-      <c r="P130" s="7" t="inlineStr">
+      <c r="P130" s="7" t="inlineStr"/>
+      <c r="Q130" s="7" t="inlineStr">
         <is>
           <t>chez-gladines</t>
         </is>
@@ -9789,7 +10151,8 @@
       <c r="O131" s="9" t="n">
         <v>2.3527</v>
       </c>
-      <c r="P131" s="9" t="inlineStr">
+      <c r="P131" s="9" t="inlineStr"/>
+      <c r="Q131" s="9" t="inlineStr">
         <is>
           <t>avant-gout</t>
         </is>
@@ -9855,7 +10218,8 @@
       <c r="O132" s="7" t="n">
         <v>2.3437</v>
       </c>
-      <c r="P132" s="7" t="inlineStr">
+      <c r="P132" s="7" t="inlineStr"/>
+      <c r="Q132" s="7" t="inlineStr">
         <is>
           <t>cite-florale</t>
         </is>
@@ -9925,7 +10289,8 @@
       <c r="O133" s="9" t="n">
         <v>2.3622</v>
       </c>
-      <c r="P133" s="9" t="inlineStr">
+      <c r="P133" s="9" t="inlineStr"/>
+      <c r="Q133" s="9" t="inlineStr">
         <is>
           <t>lao-lane-xang</t>
         </is>
@@ -9995,7 +10360,8 @@
       <c r="O134" s="7" t="n">
         <v>2.3593</v>
       </c>
-      <c r="P134" s="7" t="inlineStr">
+      <c r="P134" s="7" t="inlineStr"/>
+      <c r="Q134" s="7" t="inlineStr">
         <is>
           <t>pho-14</t>
         </is>
@@ -10065,7 +10431,8 @@
       <c r="O135" s="9" t="n">
         <v>2.3763</v>
       </c>
-      <c r="P135" s="9" t="inlineStr">
+      <c r="P135" s="9" t="inlineStr"/>
+      <c r="Q135" s="9" t="inlineStr">
         <is>
           <t>piscine-josephine-baker</t>
         </is>
@@ -10135,7 +10502,8 @@
       <c r="O136" s="7" t="n">
         <v>2.3522</v>
       </c>
-      <c r="P136" s="7" t="inlineStr">
+      <c r="P136" s="7" t="inlineStr"/>
+      <c r="Q136" s="7" t="inlineStr">
         <is>
           <t>piscine-butte-aux-cailles</t>
         </is>
@@ -10207,6 +10575,11 @@
       </c>
       <c r="P137" s="9" t="inlineStr">
         <is>
+          <t>https://www.catacombes.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q137" s="9" t="inlineStr">
+        <is>
           <t>catacombes</t>
         </is>
       </c>
@@ -10275,7 +10648,8 @@
       <c r="O138" s="7" t="n">
         <v>2.3252</v>
       </c>
-      <c r="P138" s="7" t="inlineStr">
+      <c r="P138" s="7" t="inlineStr"/>
+      <c r="Q138" s="7" t="inlineStr">
         <is>
           <t>creperie-josselin</t>
         </is>
@@ -10347,6 +10721,11 @@
       </c>
       <c r="P139" s="9" t="inlineStr">
         <is>
+          <t>https://www.lacoupole-paris.com</t>
+        </is>
+      </c>
+      <c r="Q139" s="9" t="inlineStr">
+        <is>
           <t>la-coupole</t>
         </is>
       </c>
@@ -10415,7 +10794,8 @@
       <c r="O140" s="7" t="n">
         <v>2.3289</v>
       </c>
-      <c r="P140" s="7" t="inlineStr">
+      <c r="P140" s="7" t="inlineStr"/>
+      <c r="Q140" s="7" t="inlineStr">
         <is>
           <t>le-dome</t>
         </is>
@@ -10485,7 +10865,8 @@
       <c r="O141" s="9" t="n">
         <v>2.3244</v>
       </c>
-      <c r="P141" s="9" t="inlineStr">
+      <c r="P141" s="9" t="inlineStr"/>
+      <c r="Q141" s="9" t="inlineStr">
         <is>
           <t>le-severo</t>
         </is>
@@ -10551,7 +10932,8 @@
       <c r="O142" s="7" t="n">
         <v>2.3378</v>
       </c>
-      <c r="P142" s="7" t="inlineStr">
+      <c r="P142" s="7" t="inlineStr"/>
+      <c r="Q142" s="7" t="inlineStr">
         <is>
           <t>parc-montsouris</t>
         </is>
@@ -10621,7 +11003,8 @@
       <c r="O143" s="9" t="n">
         <v>2.3207</v>
       </c>
-      <c r="P143" s="9" t="inlineStr">
+      <c r="P143" s="9" t="inlineStr"/>
+      <c r="Q143" s="9" t="inlineStr">
         <is>
           <t>pari-roller</t>
         </is>
@@ -10687,7 +11070,8 @@
       <c r="O144" s="7" t="n">
         <v>2.3187</v>
       </c>
-      <c r="P144" s="7" t="inlineStr">
+      <c r="P144" s="7" t="inlineStr"/>
+      <c r="Q144" s="7" t="inlineStr">
         <is>
           <t>rue-thermopyles</t>
         </is>
@@ -10757,7 +11141,8 @@
       <c r="O145" s="9" t="n">
         <v>2.2947</v>
       </c>
-      <c r="P145" s="9" t="inlineStr">
+      <c r="P145" s="9" t="inlineStr"/>
+      <c r="Q145" s="9" t="inlineStr">
         <is>
           <t>cafe-du-commerce</t>
         </is>
@@ -10829,6 +11214,11 @@
       </c>
       <c r="P146" s="7" t="inlineStr">
         <is>
+          <t>https://www.cordonbleu.edu/paris</t>
+        </is>
+      </c>
+      <c r="Q146" s="7" t="inlineStr">
+        <is>
           <t>cordon-bleu</t>
         </is>
       </c>
@@ -10897,7 +11287,8 @@
       <c r="O147" s="9" t="n">
         <v>2.3043</v>
       </c>
-      <c r="P147" s="9" t="inlineStr">
+      <c r="P147" s="9" t="inlineStr"/>
+      <c r="Q147" s="9" t="inlineStr">
         <is>
           <t>le-grand-pan</t>
         </is>
@@ -10968,6 +11359,11 @@
         <v>2.3219</v>
       </c>
       <c r="P148" s="7" t="inlineStr">
+        <is>
+          <t>https://www.tourmontparnasse56.com</t>
+        </is>
+      </c>
+      <c r="Q148" s="7" t="inlineStr">
         <is>
           <t>montparnasse-56</t>
         </is>
@@ -11035,6 +11431,11 @@
       </c>
       <c r="P149" s="9" t="inlineStr">
         <is>
+          <t>https://www.bourdelle.paris.fr</t>
+        </is>
+      </c>
+      <c r="Q149" s="9" t="inlineStr">
+        <is>
           <t>musee-bourdelle</t>
         </is>
       </c>
@@ -11103,7 +11504,8 @@
       <c r="O150" s="7" t="n">
         <v>2.3004</v>
       </c>
-      <c r="P150" s="7" t="inlineStr">
+      <c r="P150" s="7" t="inlineStr"/>
+      <c r="Q150" s="7" t="inlineStr">
         <is>
           <t>neige-ete</t>
         </is>
@@ -11169,7 +11571,8 @@
       <c r="O151" s="9" t="n">
         <v>2.2742</v>
       </c>
-      <c r="P151" s="9" t="inlineStr">
+      <c r="P151" s="9" t="inlineStr"/>
+      <c r="Q151" s="9" t="inlineStr">
         <is>
           <t>parc-andre-citroen</t>
         </is>
@@ -11241,6 +11644,11 @@
       </c>
       <c r="P152" s="7" t="inlineStr">
         <is>
+          <t>https://www.aquariumdeparis.com</t>
+        </is>
+      </c>
+      <c r="Q152" s="7" t="inlineStr">
+        <is>
           <t>aquarium-paris</t>
         </is>
       </c>
@@ -11309,7 +11717,8 @@
       <c r="O153" s="9" t="n">
         <v>2.2553</v>
       </c>
-      <c r="P153" s="9" t="inlineStr">
+      <c r="P153" s="9" t="inlineStr"/>
+      <c r="Q153" s="9" t="inlineStr">
         <is>
           <t>hippodrome-auteuil</t>
         </is>
@@ -11380,6 +11789,11 @@
         <v>2.2641</v>
       </c>
       <c r="P154" s="7" t="inlineStr">
+        <is>
+          <t>https://www.jardindacclimatation.fr</t>
+        </is>
+      </c>
+      <c r="Q154" s="7" t="inlineStr">
         <is>
           <t>jardin-acclimatation</t>
         </is>
@@ -11445,7 +11859,8 @@
       <c r="O155" s="9" t="n">
         <v>2.2525</v>
       </c>
-      <c r="P155" s="9" t="inlineStr">
+      <c r="P155" s="9" t="inlineStr"/>
+      <c r="Q155" s="9" t="inlineStr">
         <is>
           <t>serres-auteuil</t>
         </is>
@@ -11515,7 +11930,8 @@
       <c r="O156" s="7" t="n">
         <v>2.2717</v>
       </c>
-      <c r="P156" s="7" t="inlineStr">
+      <c r="P156" s="7" t="inlineStr"/>
+      <c r="Q156" s="7" t="inlineStr">
         <is>
           <t>la-gare</t>
         </is>
@@ -11585,7 +12001,8 @@
       <c r="O157" s="9" t="n">
         <v>2.2849</v>
       </c>
-      <c r="P157" s="9" t="inlineStr">
+      <c r="P157" s="9" t="inlineStr"/>
+      <c r="Q157" s="9" t="inlineStr">
         <is>
           <t>petit-retro</t>
         </is>
@@ -11657,6 +12074,11 @@
       </c>
       <c r="P158" s="7" t="inlineStr">
         <is>
+          <t>https://www.monsieurbleu.com</t>
+        </is>
+      </c>
+      <c r="Q158" s="7" t="inlineStr">
+        <is>
           <t>monsieur-bleu</t>
         </is>
       </c>
@@ -11725,7 +12147,8 @@
       <c r="O159" s="9" t="n">
         <v>2.2791</v>
       </c>
-      <c r="P159" s="9" t="inlineStr">
+      <c r="P159" s="9" t="inlineStr"/>
+      <c r="Q159" s="9" t="inlineStr">
         <is>
           <t>musee-contrefacon</t>
         </is>
@@ -11797,6 +12220,11 @@
       </c>
       <c r="P160" s="7" t="inlineStr">
         <is>
+          <t>https://www.museeduvinparis.com</t>
+        </is>
+      </c>
+      <c r="Q160" s="7" t="inlineStr">
+        <is>
           <t>musee-du-vin</t>
         </is>
       </c>
@@ -11867,6 +12295,11 @@
       </c>
       <c r="P161" s="9" t="inlineStr">
         <is>
+          <t>https://palaisdetokyo.com</t>
+        </is>
+      </c>
+      <c r="Q161" s="9" t="inlineStr">
+        <is>
           <t>palais-tokyo</t>
         </is>
       </c>
@@ -11937,6 +12370,11 @@
       </c>
       <c r="P162" s="7" t="inlineStr">
         <is>
+          <t>https://www.psg.fr</t>
+        </is>
+      </c>
+      <c r="Q162" s="7" t="inlineStr">
+        <is>
           <t>parc-des-princes</t>
         </is>
       </c>
@@ -12007,6 +12445,11 @@
       </c>
       <c r="P163" s="9" t="inlineStr">
         <is>
+          <t>https://www.rolandgarros.com</t>
+        </is>
+      </c>
+      <c r="Q163" s="9" t="inlineStr">
+        <is>
           <t>roland-garros</t>
         </is>
       </c>
@@ -12075,7 +12518,8 @@
       <c r="O164" s="7" t="n">
         <v>2.3132</v>
       </c>
-      <c r="P164" s="7" t="inlineStr">
+      <c r="P164" s="7" t="inlineStr"/>
+      <c r="Q164" s="7" t="inlineStr">
         <is>
           <t>coretta</t>
         </is>
@@ -12145,7 +12589,8 @@
       <c r="O165" s="9" t="n">
         <v>2.2985</v>
       </c>
-      <c r="P165" s="9" t="inlineStr">
+      <c r="P165" s="9" t="inlineStr"/>
+      <c r="Q165" s="9" t="inlineStr">
         <is>
           <t>bistrot-flaubert</t>
         </is>
@@ -12215,7 +12660,8 @@
       <c r="O166" s="7" t="n">
         <v>2.3218</v>
       </c>
-      <c r="P166" s="7" t="inlineStr">
+      <c r="P166" s="7" t="inlineStr"/>
+      <c r="Q166" s="7" t="inlineStr">
         <is>
           <t>bistrot-des-dames</t>
         </is>
@@ -12281,7 +12727,8 @@
       <c r="O167" s="9" t="n">
         <v>2.3161</v>
       </c>
-      <c r="P167" s="9" t="inlineStr">
+      <c r="P167" s="9" t="inlineStr"/>
+      <c r="Q167" s="9" t="inlineStr">
         <is>
           <t>parc-batignolles</t>
         </is>
@@ -12353,6 +12800,11 @@
       </c>
       <c r="P168" s="7" t="inlineStr">
         <is>
+          <t>https://au-lapin-agile.com</t>
+        </is>
+      </c>
+      <c r="Q168" s="7" t="inlineStr">
+        <is>
           <t>lapin-agile</t>
         </is>
       </c>
@@ -12421,7 +12873,8 @@
       <c r="O169" s="9" t="n">
         <v>2.3393</v>
       </c>
-      <c r="P169" s="9" t="inlineStr">
+      <c r="P169" s="9" t="inlineStr"/>
+      <c r="Q169" s="9" t="inlineStr">
         <is>
           <t>bouillon-pigalle</t>
         </is>
@@ -12491,7 +12944,8 @@
       <c r="O170" s="7" t="n">
         <v>2.3386</v>
       </c>
-      <c r="P170" s="7" t="inlineStr">
+      <c r="P170" s="7" t="inlineStr"/>
+      <c r="Q170" s="7" t="inlineStr">
         <is>
           <t>maison-rose</t>
         </is>
@@ -12561,7 +13015,8 @@
       <c r="O171" s="9" t="n">
         <v>2.3363</v>
       </c>
-      <c r="P171" s="9" t="inlineStr">
+      <c r="P171" s="9" t="inlineStr"/>
+      <c r="Q171" s="9" t="inlineStr">
         <is>
           <t>la-mascotte</t>
         </is>
@@ -12627,7 +13082,8 @@
       <c r="O172" s="7" t="n">
         <v>2.3446</v>
       </c>
-      <c r="P172" s="7" t="inlineStr">
+      <c r="P172" s="7" t="inlineStr"/>
+      <c r="Q172" s="7" t="inlineStr">
         <is>
           <t>recyclerie</t>
         </is>
@@ -12697,7 +13153,8 @@
       <c r="O173" s="9" t="n">
         <v>2.3355</v>
       </c>
-      <c r="P173" s="9" t="inlineStr">
+      <c r="P173" s="9" t="inlineStr"/>
+      <c r="Q173" s="9" t="inlineStr">
         <is>
           <t>coq-et-fils</t>
         </is>
@@ -12767,7 +13224,8 @@
       <c r="O174" s="7" t="n">
         <v>2.3363</v>
       </c>
-      <c r="P174" s="7" t="inlineStr">
+      <c r="P174" s="7" t="inlineStr"/>
+      <c r="Q174" s="7" t="inlineStr">
         <is>
           <t>moulin-galette</t>
         </is>
@@ -12833,7 +13291,8 @@
       <c r="O175" s="9" t="n">
         <v>2.3386</v>
       </c>
-      <c r="P175" s="9" t="inlineStr">
+      <c r="P175" s="9" t="inlineStr"/>
+      <c r="Q175" s="9" t="inlineStr">
         <is>
           <t>mur-je-taime</t>
         </is>
@@ -12899,7 +13358,8 @@
       <c r="O176" s="7" t="n">
         <v>2.337</v>
       </c>
-      <c r="P176" s="7" t="inlineStr">
+      <c r="P176" s="7" t="inlineStr"/>
+      <c r="Q176" s="7" t="inlineStr">
         <is>
           <t>tres-particulier</t>
         </is>
@@ -12971,6 +13431,11 @@
       </c>
       <c r="P177" s="9" t="inlineStr">
         <is>
+          <t>https://museedemontmartre.fr</t>
+        </is>
+      </c>
+      <c r="Q177" s="9" t="inlineStr">
+        <is>
           <t>musee-montmartre</t>
         </is>
       </c>
@@ -13039,7 +13504,8 @@
       <c r="O178" s="7" t="n">
         <v>2.343</v>
       </c>
-      <c r="P178" s="7" t="inlineStr">
+      <c r="P178" s="7" t="inlineStr"/>
+      <c r="Q178" s="7" t="inlineStr">
         <is>
           <t>puces-saint-ouen</t>
         </is>
@@ -13109,7 +13575,8 @@
       <c r="O179" s="9" t="n">
         <v>2.3363</v>
       </c>
-      <c r="P179" s="9" t="inlineStr">
+      <c r="P179" s="9" t="inlineStr"/>
+      <c r="Q179" s="9" t="inlineStr">
         <is>
           <t>studio-28</t>
         </is>
@@ -13175,7 +13642,8 @@
       <c r="O180" s="7" t="n">
         <v>2.3363</v>
       </c>
-      <c r="P180" s="7" t="inlineStr">
+      <c r="P180" s="7" t="inlineStr"/>
+      <c r="Q180" s="7" t="inlineStr">
         <is>
           <t>villa-leandre</t>
         </is>
@@ -13241,7 +13709,8 @@
       <c r="O181" s="9" t="n">
         <v>2.3811</v>
       </c>
-      <c r="P181" s="9" t="inlineStr">
+      <c r="P181" s="9" t="inlineStr"/>
+      <c r="Q181" s="9" t="inlineStr">
         <is>
           <t>butte-bergeyre</t>
         </is>
@@ -13311,7 +13780,8 @@
       <c r="O182" s="7" t="n">
         <v>2.3906</v>
       </c>
-      <c r="P182" s="7" t="inlineStr">
+      <c r="P182" s="7" t="inlineStr"/>
+      <c r="Q182" s="7" t="inlineStr">
         <is>
           <t>cinema-plein-air</t>
         </is>
@@ -13383,6 +13853,11 @@
       </c>
       <c r="P183" s="9" t="inlineStr">
         <is>
+          <t>https://www.cite-sciences.fr</t>
+        </is>
+      </c>
+      <c r="Q183" s="9" t="inlineStr">
+        <is>
           <t>cite-sciences</t>
         </is>
       </c>
@@ -13452,6 +13927,11 @@
         <v>2.3713</v>
       </c>
       <c r="P184" s="7" t="inlineStr">
+        <is>
+          <t>https://www.canauxrama.com</t>
+        </is>
+      </c>
+      <c r="Q184" s="7" t="inlineStr">
         <is>
           <t>canauxrama</t>
         </is>
@@ -13519,6 +13999,11 @@
       </c>
       <c r="P185" s="9" t="inlineStr">
         <is>
+          <t>https://www.104.fr</t>
+        </is>
+      </c>
+      <c r="Q185" s="9" t="inlineStr">
+        <is>
           <t>centquatre</t>
         </is>
       </c>
@@ -13587,7 +14072,8 @@
       <c r="O186" s="7" t="n">
         <v>2.3799</v>
       </c>
-      <c r="P186" s="7" t="inlineStr">
+      <c r="P186" s="7" t="inlineStr"/>
+      <c r="Q186" s="7" t="inlineStr">
         <is>
           <t>chapeau-melon</t>
         </is>
@@ -13659,6 +14145,11 @@
       </c>
       <c r="P187" s="9" t="inlineStr">
         <is>
+          <t>https://www.marindeaudouce.fr</t>
+        </is>
+      </c>
+      <c r="Q187" s="9" t="inlineStr">
+        <is>
           <t>marin-eau-douce</t>
         </is>
       </c>
@@ -13727,7 +14218,8 @@
       <c r="O188" s="7" t="n">
         <v>2.3886</v>
       </c>
-      <c r="P188" s="7" t="inlineStr">
+      <c r="P188" s="7" t="inlineStr"/>
+      <c r="Q188" s="7" t="inlineStr">
         <is>
           <t>mensae</t>
         </is>
@@ -13797,7 +14289,8 @@
       <c r="O189" s="9" t="n">
         <v>2.3749</v>
       </c>
-      <c r="P189" s="9" t="inlineStr">
+      <c r="P189" s="9" t="inlineStr"/>
+      <c r="Q189" s="9" t="inlineStr">
         <is>
           <t>paname-brewing</t>
         </is>
@@ -13863,7 +14356,8 @@
       <c r="O190" s="7" t="n">
         <v>2.3828</v>
       </c>
-      <c r="P190" s="7" t="inlineStr">
+      <c r="P190" s="7" t="inlineStr"/>
+      <c r="Q190" s="7" t="inlineStr">
         <is>
           <t>buttes-chaumont</t>
         </is>
@@ -13931,6 +14425,11 @@
       </c>
       <c r="P191" s="9" t="inlineStr">
         <is>
+          <t>https://www.rosabonheur.fr</t>
+        </is>
+      </c>
+      <c r="Q191" s="9" t="inlineStr">
+        <is>
           <t>rosa-bonheur</t>
         </is>
       </c>
@@ -13995,7 +14494,8 @@
       <c r="O192" s="7" t="n">
         <v>2.3933</v>
       </c>
-      <c r="P192" s="7" t="inlineStr">
+      <c r="P192" s="7" t="inlineStr"/>
+      <c r="Q192" s="7" t="inlineStr">
         <is>
           <t>pere-lachaise</t>
         </is>
@@ -14061,7 +14561,8 @@
       <c r="O193" s="9" t="n">
         <v>2.408</v>
       </c>
-      <c r="P193" s="9" t="inlineStr">
+      <c r="P193" s="9" t="inlineStr"/>
+      <c r="Q193" s="9" t="inlineStr">
         <is>
           <t>campagne-paris</t>
         </is>
@@ -14131,7 +14632,8 @@
       <c r="O194" s="7" t="n">
         <v>2.3827</v>
       </c>
-      <c r="P194" s="7" t="inlineStr">
+      <c r="P194" s="7" t="inlineStr"/>
+      <c r="Q194" s="7" t="inlineStr">
         <is>
           <t>baratin</t>
         </is>
@@ -14201,7 +14703,8 @@
       <c r="O195" s="9" t="n">
         <v>2.4046</v>
       </c>
-      <c r="P195" s="9" t="inlineStr">
+      <c r="P195" s="9" t="inlineStr"/>
+      <c r="Q195" s="9" t="inlineStr">
         <is>
           <t>allobroges</t>
         </is>
@@ -14272,6 +14775,11 @@
         <v>2.4028</v>
       </c>
       <c r="P196" s="7" t="inlineStr">
+        <is>
+          <t>https://www.mamashelter.com</t>
+        </is>
+      </c>
+      <c r="Q196" s="7" t="inlineStr">
         <is>
           <t>mama-shelter-resto</t>
         </is>
@@ -14337,14 +14845,15 @@
       <c r="O197" s="9" t="n">
         <v>2.3788</v>
       </c>
-      <c r="P197" s="9" t="inlineStr">
+      <c r="P197" s="9" t="inlineStr"/>
+      <c r="Q197" s="9" t="inlineStr">
         <is>
           <t>rue-denoyez</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P197"/>
+  <autoFilter ref="A1:Q197"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>